<commit_message>
[Added testing file docs]
Added test cases for login process
</commit_message>
<xml_diff>
--- a/docs/User Test Case.xlsx
+++ b/docs/User Test Case.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>TestID</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Pass/Fail</t>
   </si>
   <si>
-    <t>Test_01</t>
+    <t>RegistrationTest_01</t>
   </si>
   <si>
     <t>Registration with valid details</t>
@@ -46,7 +46,7 @@
     <t>User should be registered successfully, no errors</t>
   </si>
   <si>
-    <t>Test_02</t>
+    <t>RegistrationTest_02</t>
   </si>
   <si>
     <t>Registration with invalid name</t>
@@ -61,7 +61,7 @@
     <t>Error message: “Invalid name. Please use letters only.”</t>
   </si>
   <si>
-    <t>Test_03</t>
+    <t>RegistrationTest_03</t>
   </si>
   <si>
     <t>Registration with invalid email</t>
@@ -76,32 +76,41 @@
     <t>Error message: “Invalid email format.”</t>
   </si>
   <si>
-    <t>Test_04</t>
+    <t>RegistrationTest_04</t>
   </si>
   <si>
     <t>Registration with invalid role</t>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Name: John DoeEmail: </t>
+      <rPr>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve">Name: John Doe
+Email: </t>
     </r>
     <r>
       <rPr>
         <color rgb="FF1155CC"/>
+        <sz val="11.0"/>
         <u/>
       </rPr>
-      <t>john@example.com</t>
+      <t xml:space="preserve">john@example.com
+</t>
     </r>
     <r>
-      <rPr/>
-      <t>Role: Adminnn (not in dropdown)Password: StrongP@ss</t>
+      <rPr>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Role: Adminnn (not in dropdown)
+Password: StrongP@ss</t>
     </r>
   </si>
   <si>
     <t>Error message: “Invalid role selected.”</t>
   </si>
   <si>
-    <t>Test_05</t>
+    <t>RegistrationTest_05</t>
   </si>
   <si>
     <t>Registration with invalid password</t>
@@ -114,6 +123,128 @@
   </si>
   <si>
     <t>Error message: “Password must be at least 8 characters, include letters and numbers.”</t>
+  </si>
+  <si>
+    <t>LoginTest_01</t>
+  </si>
+  <si>
+    <t>Login with valid email and password</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve">Email: </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t xml:space="preserve">john@example.com
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Password: StrongP@ss</t>
+    </r>
+  </si>
+  <si>
+    <t>User is successfully logged in and redirected to dashboard</t>
+  </si>
+  <si>
+    <t>LoginTest_02</t>
+  </si>
+  <si>
+    <t>Login with invalid email format</t>
+  </si>
+  <si>
+    <t>Email: johnexample.com
+Password: StrongP@ss</t>
+  </si>
+  <si>
+    <t>Error message – “Invalid email format.”</t>
+  </si>
+  <si>
+    <t>LoginTest_03</t>
+  </si>
+  <si>
+    <t>Login with invalid password format</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve">Email: </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t xml:space="preserve">john@example.com
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Password: 12345</t>
+    </r>
+  </si>
+  <si>
+    <t>Error message – “Incorrect password.”</t>
+  </si>
+  <si>
+    <t>LoginTest_04</t>
+  </si>
+  <si>
+    <t>Login with blank fields</t>
+  </si>
+  <si>
+    <t>Email: [empty]
+Password: [empty]</t>
+  </si>
+  <si>
+    <t>Error message – “Email and password are required.”</t>
+  </si>
+  <si>
+    <t>LoginTest_05</t>
+  </si>
+  <si>
+    <t>Login with valid email but wrong password</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve">Email: </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <sz val="11.0"/>
+        <u/>
+      </rPr>
+      <t xml:space="preserve">john@example.com
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.0"/>
+      </rPr>
+      <t>Password: WrongPass123</t>
+    </r>
+  </si>
+  <si>
+    <t>Error message – “Invalid credentials.”</t>
   </si>
 </sst>
 </file>
@@ -128,18 +259,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="13.0"/>
+      <b/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="11.0"/>
       <color rgb="FF0000FF"/>
     </font>
   </fonts>
@@ -182,7 +316,7 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -412,7 +546,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="18.88"/>
+    <col customWidth="1" min="1" max="6" width="25.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -423,7 +557,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2">
+    <row r="2" ht="60.0" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -443,7 +577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="60.0" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -459,7 +593,7 @@
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
     </row>
-    <row r="4">
+    <row r="4" ht="60.0" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
@@ -475,7 +609,7 @@
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5">
+    <row r="5" ht="60.0" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -491,7 +625,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6">
+    <row r="6" ht="60.0" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -507,7 +641,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7">
+    <row r="7" ht="60.0" customHeight="1">
       <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
@@ -523,45 +657,85 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
+    <row r="8" ht="60.0" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" ht="60.0" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" ht="60.0" customHeight="1">
+      <c r="A10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" ht="60.0" customHeight="1">
+      <c r="A11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" ht="60.0" customHeight="1">
+      <c r="A12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
     </row>
     <row r="13">
       <c r="A13" s="1"/>
@@ -8443,26 +8617,13 @@
       <c r="E997" s="1"/>
       <c r="F997" s="1"/>
     </row>
-    <row r="998">
-      <c r="A998" s="1"/>
-      <c r="B998" s="1"/>
-      <c r="C998" s="1"/>
-      <c r="D998" s="1"/>
-      <c r="E998" s="1"/>
-      <c r="F998" s="1"/>
-    </row>
-    <row r="999">
-      <c r="A999" s="1"/>
-      <c r="B999" s="1"/>
-      <c r="C999" s="1"/>
-      <c r="D999" s="1"/>
-      <c r="E999" s="1"/>
-      <c r="F999" s="1"/>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C6"/>
+    <hyperlink r:id="rId2" ref="C8"/>
+    <hyperlink r:id="rId3" ref="C10"/>
+    <hyperlink r:id="rId4" ref="C12"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
New, More Comprehensive, Test Cases
</commit_message>
<xml_diff>
--- a/docs/User Test Case.xlsx
+++ b/docs/User Test Case.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dell/Documents/Documents/Work/Monash/Year 2/FIT2101/Project/MA_Thursday5pm_Team3/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A778F64-8A72-DF45-9B6F-C49B2E158D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA7DEF0-9BB5-1E47-B0BB-6AB1D354201F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="60">
   <si>
     <t>TestID</t>
   </si>
@@ -46,28 +46,16 @@
     <t>Registration with valid details</t>
   </si>
   <si>
-    <t>Name: John Doe
-Email: john@example.com
-Role: Student
-Password: StrongP@ss</t>
-  </si>
-  <si>
     <t>User should be registered successfully, no errors</t>
   </si>
   <si>
     <t>RegistrationTest_02</t>
   </si>
   <si>
-    <t>Registration with invalid name</t>
-  </si>
-  <si>
     <t>Error message: “Invalid name. Please use letters only.”</t>
   </si>
   <si>
     <t>RegistrationTest_03</t>
-  </si>
-  <si>
-    <t>Registration with invalid email</t>
   </si>
   <si>
     <t>Error message: “Invalid email format.”</t>
@@ -77,15 +65,6 @@
   </si>
   <si>
     <t>RegistrationTest_05</t>
-  </si>
-  <si>
-    <t>Registration with invalid password</t>
-  </si>
-  <si>
-    <t>Name: John Doe
-Email: john@example.com
-Role: Student
-Password: 123 (too short, missing complexity)</t>
   </si>
   <si>
     <t>Error message: “Password must be at least 8 characters, include letters and numbers.”</t>
@@ -130,9 +109,6 @@
   </si>
   <si>
     <t>LoginTest_02</t>
-  </si>
-  <si>
-    <t>Login with invalid email format</t>
   </si>
   <si>
     <t>Email: johnexample.com
@@ -237,47 +213,94 @@
     <t>RegistrationTest_07</t>
   </si>
   <si>
-    <t>Registration with missing email</t>
-  </si>
-  <si>
     <t>Registration where two password checkboxes don't match</t>
-  </si>
-  <si>
-    <t>Name: John Doe
-Email: john@example.com
-Role: Student
-Password: StrongP@ass
-Confirm Password: StangP@ass</t>
   </si>
   <si>
     <t>Registration with invalid title</t>
   </si>
   <si>
-    <t>Error message: “Invalid title selected. Please use letters only.”</t>
-  </si>
-  <si>
     <t>RegistrationTest_08</t>
   </si>
   <si>
-    <t>Name: John Doe
+    <t>Error message: "Password and Confirm password don't match!"</t>
+  </si>
+  <si>
+    <t>Registration with invalid or missing email</t>
+  </si>
+  <si>
+    <t>Registration with invalid or missing password</t>
+  </si>
+  <si>
+    <t>Registration with invalid or missing name</t>
+  </si>
+  <si>
+    <t>Login with invalid or missing email format</t>
+  </si>
+  <si>
+    <t>RegistrationTest_09</t>
+  </si>
+  <si>
+    <t>RegistrationTest_10</t>
+  </si>
+  <si>
+    <t>First Name: John
+Last Name: Doe
+Email: john@example.com
+Role: Student
+Password: StrongP@ss</t>
+  </si>
+  <si>
+    <t>First Name: John
+Last Name: Doe
 Email: john@example.com
 Role: [Teacher/Admin]
 Title: Professor
 Password: StrongP@ss</t>
   </si>
   <si>
-    <t>Name: 1234
+    <t>First Name: 1234
+Last Name: 5678
 Email: john@example.com
 Role: [Student/Teacher/Admin]
 Title: Mr
 Password: StrongP@ss</t>
   </si>
   <si>
-    <t>Name: John Doe
+    <t>First Name: Hello
+Last Name: [blank]
+Email: john@example.com
+Role: [Student/Teacher/Admin]
+Title: Mr
+Password: StrongP@ss</t>
+  </si>
+  <si>
+    <t>First Name: John
+Last Name: Doe
 Email: johnexample.com
 Role:  [Student/Teacher/Admin]
 Title: Sir
 Password: StrongP@ss</t>
+  </si>
+  <si>
+    <t>Error message: “Invalid name. Please use letters only.” or "[First Name/Last Name] required"</t>
+  </si>
+  <si>
+    <t>First Name: John
+Last Name: Doe
+Email: [blank]
+Role:  [Student/Teacher/Admin]
+Title: Sir
+Password: StrongP@ss</t>
+  </si>
+  <si>
+    <t>Error message: “Invalid email format.” or "Email required"</t>
+  </si>
+  <si>
+    <t>First Name: John
+Last Name: Doe
+Email: john@example.com
+Role: Student
+Password: 123 (too short, missing complexity)</t>
   </si>
   <si>
     <r>
@@ -286,7 +309,8 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Name: John Doe
+      <t xml:space="preserve">First Name: John
+Last Name: Doe
 Email: </t>
     </r>
     <r>
@@ -312,13 +336,22 @@
     </r>
   </si>
   <si>
-    <t>Name: John Doe
-Email: 
-Role: Student
-Password: 123</t>
+    <t>Error message: “Invalid title name. Please use letters only.”</t>
   </si>
   <si>
-    <t>Error message: "Password and Confirm password don't match!"</t>
+    <t>First Name: John
+Last Name: Doe
+Email: john@example.com
+Role: Student
+Password: StrongP@ass
+Confirm Password: StangP@ass</t>
+  </si>
+  <si>
+    <t>First Name: John
+Last Name: Doe
+Email: john@example.com
+Role: Student
+Password: [missing]</t>
   </si>
 </sst>
 </file>
@@ -646,7 +679,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F1000"/>
+  <dimension ref="A1:F1002"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="6" width="25.1640625" customWidth="1"/>
@@ -680,7 +713,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:6" ht="75" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -688,221 +721,237 @@
         <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" ht="79" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:6" ht="90" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="1:6" ht="89" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:6" ht="105" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="1:6" ht="94" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:6" ht="105" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:6" ht="83" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:6" ht="105" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>52</v>
+      <c r="C7" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:6" ht="77" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:6" ht="105" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="C8" s="3" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:6" ht="78" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:6" ht="90" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>53</v>
+      <c r="C9" s="4" t="s">
+        <v>56</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="1:6" ht="84" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:6" ht="75" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:6" ht="90" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>23</v>
+      <c r="C11" s="3" t="s">
+        <v>55</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:6" ht="105" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" ht="14" x14ac:dyDescent="0.15">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" ht="14" x14ac:dyDescent="0.15">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+    <row r="16" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6" ht="14" x14ac:dyDescent="0.15">
       <c r="A18" s="1"/>
@@ -8768,13 +8817,29 @@
       <c r="E1000" s="1"/>
       <c r="F1000" s="1"/>
     </row>
+    <row r="1001" spans="1:6" ht="14" x14ac:dyDescent="0.15">
+      <c r="A1001" s="1"/>
+      <c r="B1001" s="1"/>
+      <c r="C1001" s="1"/>
+      <c r="D1001" s="1"/>
+      <c r="E1001" s="1"/>
+      <c r="F1001" s="1"/>
+    </row>
+    <row r="1002" spans="1:6" ht="14" x14ac:dyDescent="0.15">
+      <c r="A1002" s="1"/>
+      <c r="B1002" s="1"/>
+      <c r="C1002" s="1"/>
+      <c r="D1002" s="1"/>
+      <c r="E1002" s="1"/>
+      <c r="F1002" s="1"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C7" r:id="rId1" display="Name: John Doe_x000a_Email: john@example.com_x000a_Role: Adminnn (not in dropdown)_x000a_Password: StrongP@ss" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="C11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="C13" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="C15" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="C9" r:id="rId1" display="Name: John Doe_x000a_Email: john@example.com_x000a_Role: Adminnn (not in dropdown)_x000a_Password: StrongP@ss" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C13" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="C15" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="C17" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
-Filled in user test case for login and register
</commit_message>
<xml_diff>
--- a/docs/User Test Case.xlsx
+++ b/docs/User Test Case.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
   <si>
     <t>TestID</t>
   </si>
@@ -40,10 +40,17 @@
     <t>Name: John Doe
 Email: john@example.com
 Role: Student
-Password: StrongP@ss</t>
+Password: StrongP@ss
+Token: STUDENTCB6TL</t>
   </si>
   <si>
     <t>User should be registered successfully, no errors</t>
+  </si>
+  <si>
+    <t>User registered succesfully, no errors</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
   <si>
     <t>RegistrationTest_02</t>
@@ -79,40 +86,6 @@
     <t>RegistrationTest_04</t>
   </si>
   <si>
-    <t>Registration with invalid role</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">Name: John Doe
-Email: </t>
-    </r>
-    <r>
-      <rPr>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t xml:space="preserve">john@example.com
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Role: Adminnn (not in dropdown)
-Password: StrongP@ss</t>
-    </r>
-  </si>
-  <si>
-    <t>Error message: “Invalid role selected.”</t>
-  </si>
-  <si>
-    <t>RegistrationTest_05</t>
-  </si>
-  <si>
     <t>Registration with invalid password</t>
   </si>
   <si>
@@ -122,7 +95,7 @@
 Password: 123 (too short, missing complexity)</t>
   </si>
   <si>
-    <t>Error message: “Password must be at least 8 characters, include letters and numbers.”</t>
+    <t>Cannot create user! FirebaseError: Firebase: Password should be at least 6 characters (auth/weak-password).</t>
   </si>
   <si>
     <t>LoginTest_01</t>
@@ -199,7 +172,7 @@
     </r>
   </si>
   <si>
-    <t>Error message – “Incorrect password.”</t>
+    <t>Error message – “Cannot sign in user! FirebaseError: Firebase: Error (auth/invalid-login-credentials).”</t>
   </si>
   <si>
     <t>LoginTest_04</t>
@@ -212,7 +185,7 @@
 Password: [empty]</t>
   </si>
   <si>
-    <t>Error message – “Email and password are required.”</t>
+    <t>Error message – “Cannot sign in user! FirebaseError: Firebase: Error (auth/invalid-login-credentials)..”</t>
   </si>
   <si>
     <t>LoginTest_05</t>
@@ -242,9 +215,6 @@
       </rPr>
       <t>Password: WrongPass123</t>
     </r>
-  </si>
-  <si>
-    <t>Error message – “Invalid credentials.”</t>
   </si>
 </sst>
 </file>
@@ -311,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -331,6 +301,9 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -577,7 +550,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="60.0" customHeight="1">
+    <row r="3" ht="75.0" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -590,155 +563,183 @@
       <c r="D3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-    </row>
-    <row r="4" ht="60.0" customHeight="1">
-      <c r="A4" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4" t="s">
+    </row>
+    <row r="4" ht="75.0" customHeight="1">
+      <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5" ht="60.0" customHeight="1">
-      <c r="A5" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" ht="75.0" customHeight="1">
+      <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-    </row>
-    <row r="6" ht="60.0" customHeight="1">
-      <c r="A6" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="E5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" ht="75.0" customHeight="1">
+      <c r="A6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-    </row>
-    <row r="7" ht="60.0" customHeight="1">
-      <c r="A7" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="E6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" ht="75.0" customHeight="1">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+    </row>
+    <row r="8" ht="75.0" customHeight="1">
+      <c r="A8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-    </row>
-    <row r="8" ht="60.0" customHeight="1">
-      <c r="A8" s="3" t="s">
+      <c r="C8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="E8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" ht="75.0" customHeight="1">
+      <c r="A9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-    </row>
-    <row r="9" ht="60.0" customHeight="1">
-      <c r="A9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="E9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" ht="75.0" customHeight="1">
+      <c r="A10" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-    </row>
-    <row r="10" ht="60.0" customHeight="1">
-      <c r="A10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="E10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" ht="75.0" customHeight="1">
+      <c r="A11" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="B11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-    </row>
-    <row r="11" ht="60.0" customHeight="1">
-      <c r="A11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="E11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" ht="75.0" customHeight="1">
+      <c r="A12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-    </row>
-    <row r="12" ht="60.0" customHeight="1">
-      <c r="A12" s="3" t="s">
+      <c r="C12" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>43</v>
+      <c r="D12" s="3" t="s">
+        <v>35</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>44</v>
+      <c r="E12" s="3" t="s">
+        <v>39</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>45</v>
+      <c r="F12" s="3" t="s">
+        <v>11</v>
       </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
     </row>
     <row r="13">
-      <c r="A13" s="1"/>
+      <c r="A13" s="7"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -8619,11 +8620,10 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C6"/>
-    <hyperlink r:id="rId2" ref="C8"/>
-    <hyperlink r:id="rId3" ref="C10"/>
-    <hyperlink r:id="rId4" ref="C12"/>
+    <hyperlink r:id="rId1" ref="C8"/>
+    <hyperlink r:id="rId2" ref="C10"/>
+    <hyperlink r:id="rId3" ref="C12"/>
   </hyperlinks>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>